<commit_message>
travel-schedule-excel: Schedule sheet only, drop Hotel/Visitors
build_master.py에서 Hotel/Visitors 시트 생성 제거, 마스터 xlsx 재생성(Schedule 단일 시트), SKILL.md 문서 일치 수정.
</commit_message>
<xml_diff>
--- a/travel-schedule-excel/_templates/business_trip_master.xlsx
+++ b/travel-schedule-excel/_templates/business_trip_master.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hotel" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visitors" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,30 +466,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>